<commit_message>
fix: Module2 파이프라인 정리 및 TpgCtrlTop enable 신호 CDC 동기화 추가
- Module2: 미정의 신호(H_dta, En_D_1D, H_sum_1D 등) 참조 오류 수정, 2단 출력 레지스터 구조로 정리
- TpgCtrlTop: IfClk 도메인의 M1_en/M2_en을 SysClk 도메인으로 2FF 동기화(M1_en_sync/M2_en_sync)한 뒤 Module1/2에 연결
- EEPROM.drawio를 Total/TpgCtrlTop/TB Block Diagram으로 분리, SysClk 타이밍 계산·비트차트 문서 추가, 체크리스트 갱신
</commit_message>
<xml_diff>
--- a/참고사항/24LC256_체크리스트_1.xlsx
+++ b/참고사항/24LC256_체크리스트_1.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BLUE\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BLUE\work\VHDL\FSM_EEPROM\참고사항\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24690" windowHeight="9960" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23460" windowHeight="9960" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="체크리스트" sheetId="1" r:id="rId1"/>
@@ -3379,10 +3379,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3431,6 +3429,11 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -3580,7 +3583,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3707,7 +3709,7 @@
                   <c:v>0.88888888888888884</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3746,11 +3748,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="1629831552"/>
-        <c:axId val="1629840256"/>
+        <c:axId val="534903520"/>
+        <c:axId val="534902432"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1629831552"/>
+        <c:axId val="534903520"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3782,7 +3784,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -3818,7 +3819,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1629840256"/>
+        <c:crossAx val="534902432"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3826,7 +3827,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1629840256"/>
+        <c:axId val="534902432"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3868,7 +3869,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -3904,7 +3904,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1629831552"/>
+        <c:crossAx val="534903520"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3917,7 +3917,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4227,7 +4226,7 @@
     <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" customWidth="1"/>
     <col min="5" max="5" width="83.5703125" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
@@ -4235,1145 +4234,1145 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.75" customHeight="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="27">
-      <c r="A2" s="5">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="3">
         <v>0</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6" t="s">
+      <c r="D2" s="4"/>
+      <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="6">
         <v>46269</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="4" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="27">
-      <c r="A3" s="5">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="3">
         <v>0</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6" t="s">
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="6">
         <v>46269</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="17" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="27">
-      <c r="A4" s="5">
+    <row r="4" spans="1:8">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="3">
         <v>0</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="6">
         <v>46269</v>
       </c>
-      <c r="H4" s="6"/>
+      <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="5">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="3">
         <v>0</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6" t="s">
+      <c r="D5" s="4"/>
+      <c r="E5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="6">
         <v>46269</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="18" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="27">
-      <c r="A6" s="5">
+    <row r="6" spans="1:8">
+      <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="3">
         <v>0</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6" t="s">
+      <c r="D6" s="4"/>
+      <c r="E6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="6">
         <v>46269</v>
       </c>
-      <c r="H6" s="6"/>
+      <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" ht="27">
-      <c r="A7" s="5">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="3">
         <v>1</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="6">
         <v>46269</v>
       </c>
-      <c r="H7" s="9"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8" ht="27">
-      <c r="A8" s="5">
+      <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="3">
         <v>1</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="6">
         <v>46269</v>
       </c>
-      <c r="H8" s="9"/>
+      <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8" ht="27">
-      <c r="A9" s="5">
+      <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="3">
         <v>1</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="6">
         <v>46269</v>
       </c>
-      <c r="H9" s="9"/>
+      <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:8" ht="27">
-      <c r="A10" s="5">
+      <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="6">
         <v>46269</v>
       </c>
-      <c r="H10" s="9"/>
+      <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:8" ht="27">
-      <c r="A11" s="5">
+      <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="3">
         <v>1</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="6">
         <v>46269</v>
       </c>
-      <c r="H11" s="9"/>
+      <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:8" ht="27">
-      <c r="A12" s="5">
+      <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="3">
         <v>1</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="6">
         <v>46269</v>
       </c>
-      <c r="H12" s="9"/>
+      <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:8" ht="27">
-      <c r="A13" s="5">
+      <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="3">
         <v>1</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="8"/>
-      <c r="H13" s="9"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:8" ht="27">
-      <c r="A14" s="5">
+      <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="3">
         <v>1</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="6">
         <v>46269</v>
       </c>
-      <c r="H14" s="9"/>
+      <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:8" ht="27">
-      <c r="A15" s="5">
+      <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="3">
         <v>1</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="6">
         <v>46269</v>
       </c>
-      <c r="H15" s="9"/>
+      <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:8" ht="27">
-      <c r="A16" s="5">
+      <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="3">
         <v>2</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="9"/>
-      <c r="E16" s="6" t="s">
+      <c r="D16" s="7"/>
+      <c r="E16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="6"/>
+      <c r="H16" s="7"/>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3">
+        <v>2</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="6"/>
+      <c r="H17" s="7"/>
+    </row>
+    <row r="18" spans="1:8" ht="27">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3">
+        <v>2</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="6"/>
+      <c r="H18" s="7"/>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3">
+        <v>2</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="7"/>
+      <c r="E19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="6"/>
+      <c r="H19" s="7"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3">
+        <v>2</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20" s="6"/>
+      <c r="H20" s="7"/>
+    </row>
+    <row r="21" spans="1:8" ht="27">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3">
+        <v>3</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="G16" s="8"/>
-      <c r="H16" s="9"/>
-    </row>
-    <row r="17" spans="1:8" ht="27">
-      <c r="A17" s="5">
-        <v>16</v>
-      </c>
-      <c r="B17" s="5">
-        <v>2</v>
-      </c>
-      <c r="C17" s="6" t="s">
+      <c r="G21" s="6"/>
+      <c r="H21" s="7"/>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3">
+        <v>3</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G22" s="6"/>
+      <c r="H22" s="7"/>
+    </row>
+    <row r="23" spans="1:8" ht="27">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3">
+        <v>3</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G23" s="6"/>
+      <c r="H23" s="7"/>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3">
+        <v>3</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" s="6"/>
+      <c r="H24" s="7"/>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3">
+        <v>3</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="7"/>
+      <c r="E25" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G25" s="6"/>
+      <c r="H25" s="7"/>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3">
+        <v>4</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="7"/>
+      <c r="E26" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" s="6"/>
+      <c r="H26" s="7"/>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3">
+        <v>4</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="7"/>
+      <c r="E27" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G27" s="6"/>
+      <c r="H27" s="7"/>
+    </row>
+    <row r="28" spans="1:8" ht="27">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3">
+        <v>4</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="7"/>
+      <c r="E28" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G28" s="6"/>
+      <c r="H28" s="7"/>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="D17" s="9"/>
-      <c r="E17" s="6" t="s">
+      <c r="B29" s="3">
+        <v>4</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="7"/>
+      <c r="E29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G29" s="6"/>
+      <c r="H29" s="7"/>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="3">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3">
+        <v>4</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="7"/>
+      <c r="E30" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G30" s="6"/>
+      <c r="H30" s="7"/>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="3">
         <v>30</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="B31" s="3">
+        <v>5</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F31" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G17" s="8"/>
-      <c r="H17" s="9"/>
-    </row>
-    <row r="18" spans="1:8" ht="27">
-      <c r="A18" s="5">
-        <v>17</v>
-      </c>
-      <c r="B18" s="5">
-        <v>2</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9" t="s">
+      <c r="G31" s="6"/>
+      <c r="H31" s="7"/>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="3">
         <v>31</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="B32" s="3">
+        <v>5</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D32" s="7"/>
+      <c r="E32" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F32" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="8"/>
-      <c r="H18" s="9"/>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="5">
-        <v>18</v>
-      </c>
-      <c r="B19" s="5">
-        <v>2</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="9"/>
-      <c r="E19" s="6" t="s">
+      <c r="G32" s="6"/>
+      <c r="H32" s="7"/>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="3">
         <v>32</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="B33" s="3">
+        <v>5</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D33" s="7"/>
+      <c r="E33" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F33" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G19" s="8"/>
-      <c r="H19" s="9"/>
-    </row>
-    <row r="20" spans="1:8" ht="27">
-      <c r="A20" s="5">
-        <v>19</v>
-      </c>
-      <c r="B20" s="5">
-        <v>2</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9" t="s">
+      <c r="G33" s="6"/>
+      <c r="H33" s="7"/>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="3">
         <v>33</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="B34" s="3">
+        <v>5</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F34" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="8"/>
-      <c r="H20" s="9"/>
-    </row>
-    <row r="21" spans="1:8" ht="27">
-      <c r="A21" s="5">
-        <v>20</v>
-      </c>
-      <c r="B21" s="5">
-        <v>3</v>
-      </c>
-      <c r="C21" s="6" t="s">
+      <c r="G34" s="6"/>
+      <c r="H34" s="7"/>
+    </row>
+    <row r="35" spans="1:8" ht="27">
+      <c r="A35" s="3">
         <v>34</v>
       </c>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9" t="s">
+      <c r="B35" s="3">
+        <v>6</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G35" s="6"/>
+      <c r="H35" s="7"/>
+    </row>
+    <row r="36" spans="1:8" ht="27">
+      <c r="A36" s="3">
         <v>35</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="B36" s="3">
+        <v>6</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F36" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G21" s="8"/>
-      <c r="H21" s="9"/>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="5">
-        <v>21</v>
-      </c>
-      <c r="B22" s="5">
-        <v>3</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9" t="s">
+      <c r="G36" s="6"/>
+      <c r="H36" s="7"/>
+    </row>
+    <row r="37" spans="1:8" ht="27">
+      <c r="A37" s="3">
         <v>36</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="B37" s="3">
+        <v>6</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F37" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="8"/>
-      <c r="H22" s="9"/>
-    </row>
-    <row r="23" spans="1:8" ht="27">
-      <c r="A23" s="5">
-        <v>22</v>
-      </c>
-      <c r="B23" s="5">
-        <v>3</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9" t="s">
+      <c r="G37" s="6"/>
+      <c r="H37" s="7"/>
+    </row>
+    <row r="38" spans="1:8" ht="27">
+      <c r="A38" s="3">
         <v>37</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="B38" s="3">
+        <v>6</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F38" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G23" s="8"/>
-      <c r="H23" s="9"/>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" s="5">
-        <v>23</v>
-      </c>
-      <c r="B24" s="5">
-        <v>3</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9" t="s">
+      <c r="G38" s="6"/>
+      <c r="H38" s="7"/>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="3">
         <v>38</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="B39" s="3">
+        <v>7</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="7"/>
+      <c r="E39" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F39" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="8"/>
-      <c r="H24" s="9"/>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="5">
-        <v>24</v>
-      </c>
-      <c r="B25" s="5">
-        <v>3</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D25" s="9"/>
-      <c r="E25" s="6" t="s">
+      <c r="G39" s="6"/>
+      <c r="H39" s="7"/>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="3">
         <v>39</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="B40" s="3">
+        <v>7</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D40" s="7"/>
+      <c r="E40" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F40" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G25" s="8"/>
-      <c r="H25" s="9"/>
-    </row>
-    <row r="26" spans="1:8" ht="27">
-      <c r="A26" s="5">
-        <v>25</v>
-      </c>
-      <c r="B26" s="5">
-        <v>4</v>
-      </c>
-      <c r="C26" s="9" t="s">
+      <c r="G40" s="6"/>
+      <c r="H40" s="7"/>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="3">
         <v>40</v>
       </c>
-      <c r="D26" s="9"/>
-      <c r="E26" s="6" t="s">
+      <c r="B41" s="3">
+        <v>7</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D41" s="7"/>
+      <c r="E41" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G41" s="6"/>
+      <c r="H41" s="7"/>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="3">
         <v>41</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="B42" s="3">
+        <v>7</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D42" s="7"/>
+      <c r="E42" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F42" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G26" s="8"/>
-      <c r="H26" s="9"/>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" s="5">
-        <v>26</v>
-      </c>
-      <c r="B27" s="5">
-        <v>4</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D27" s="9"/>
-      <c r="E27" s="6" t="s">
+      <c r="G42" s="6"/>
+      <c r="H42" s="7"/>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" s="3">
         <v>42</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="B43" s="3">
+        <v>7</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D43" s="7"/>
+      <c r="E43" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F43" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G27" s="8"/>
-      <c r="H27" s="9"/>
-    </row>
-    <row r="28" spans="1:8" ht="27">
-      <c r="A28" s="5">
-        <v>27</v>
-      </c>
-      <c r="B28" s="5">
-        <v>4</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" s="9"/>
-      <c r="E28" s="6" t="s">
+      <c r="G43" s="6"/>
+      <c r="H43" s="7"/>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" s="3">
         <v>43</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="B44" s="3">
+        <v>8</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F44" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G28" s="8"/>
-      <c r="H28" s="9"/>
-    </row>
-    <row r="29" spans="1:8">
-      <c r="A29" s="5">
-        <v>28</v>
-      </c>
-      <c r="B29" s="5">
-        <v>4</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" s="9"/>
-      <c r="E29" s="6" t="s">
+      <c r="G44" s="6"/>
+      <c r="H44" s="7"/>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="3">
         <v>44</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="B45" s="3">
+        <v>8</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D45" s="7"/>
+      <c r="E45" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F45" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G29" s="8"/>
-      <c r="H29" s="9"/>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="5">
-        <v>29</v>
-      </c>
-      <c r="B30" s="5">
-        <v>4</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D30" s="9"/>
-      <c r="E30" s="6" t="s">
+      <c r="G45" s="6"/>
+      <c r="H45" s="7"/>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" s="3">
         <v>45</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="B46" s="3">
+        <v>8</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D46" s="7"/>
+      <c r="E46" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F46" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G30" s="8"/>
-      <c r="H30" s="9"/>
-    </row>
-    <row r="31" spans="1:8">
-      <c r="A31" s="5">
-        <v>30</v>
-      </c>
-      <c r="B31" s="5">
-        <v>5</v>
-      </c>
-      <c r="C31" s="9" t="s">
+      <c r="G46" s="6"/>
+      <c r="H46" s="7"/>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" s="3">
         <v>46</v>
       </c>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9" t="s">
+      <c r="B47" s="3">
+        <v>9</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D47" s="7"/>
+      <c r="E47" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G47" s="6"/>
+      <c r="H47" s="7"/>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" s="3">
         <v>47</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="B48" s="3">
+        <v>9</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D48" s="7"/>
+      <c r="E48" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F48" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G31" s="8"/>
-      <c r="H31" s="9"/>
-    </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="5">
-        <v>31</v>
-      </c>
-      <c r="B32" s="5">
-        <v>5</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D32" s="9"/>
-      <c r="E32" s="6" t="s">
+      <c r="G48" s="6"/>
+      <c r="H48" s="7"/>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="3">
         <v>48</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="B49" s="3">
+        <v>10</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D49" s="7"/>
+      <c r="E49" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F49" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G32" s="8"/>
-      <c r="H32" s="9"/>
-    </row>
-    <row r="33" spans="1:8">
-      <c r="A33" s="5">
-        <v>32</v>
-      </c>
-      <c r="B33" s="5">
-        <v>5</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D33" s="9"/>
-      <c r="E33" s="6" t="s">
+      <c r="G49" s="6"/>
+      <c r="H49" s="7"/>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="3">
         <v>49</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="B50" s="3">
+        <v>10</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D50" s="7"/>
+      <c r="E50" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F50" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G33" s="8"/>
-      <c r="H33" s="9"/>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="5">
-        <v>33</v>
-      </c>
-      <c r="B34" s="5">
-        <v>5</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9" t="s">
+      <c r="G50" s="6"/>
+      <c r="H50" s="7"/>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" s="3">
         <v>50</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="B51" s="3">
+        <v>10</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D51" s="7"/>
+      <c r="E51" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F51" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G34" s="8"/>
-      <c r="H34" s="9"/>
-    </row>
-    <row r="35" spans="1:8" ht="27">
-      <c r="A35" s="5">
-        <v>34</v>
-      </c>
-      <c r="B35" s="5">
-        <v>6</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G35" s="8"/>
-      <c r="H35" s="9"/>
-    </row>
-    <row r="36" spans="1:8" ht="27">
-      <c r="A36" s="5">
-        <v>35</v>
-      </c>
-      <c r="B36" s="5">
-        <v>6</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F36" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G36" s="8"/>
-      <c r="H36" s="9"/>
-    </row>
-    <row r="37" spans="1:8" ht="27">
-      <c r="A37" s="5">
-        <v>36</v>
-      </c>
-      <c r="B37" s="5">
-        <v>6</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G37" s="8"/>
-      <c r="H37" s="9"/>
-    </row>
-    <row r="38" spans="1:8" ht="27">
-      <c r="A38" s="5">
-        <v>37</v>
-      </c>
-      <c r="B38" s="5">
-        <v>6</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G38" s="8"/>
-      <c r="H38" s="9"/>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" s="5">
-        <v>38</v>
-      </c>
-      <c r="B39" s="5">
-        <v>7</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D39" s="9"/>
-      <c r="E39" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G39" s="8"/>
-      <c r="H39" s="9"/>
-    </row>
-    <row r="40" spans="1:8">
-      <c r="A40" s="5">
-        <v>39</v>
-      </c>
-      <c r="B40" s="5">
-        <v>7</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D40" s="9"/>
-      <c r="E40" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G40" s="8"/>
-      <c r="H40" s="9"/>
-    </row>
-    <row r="41" spans="1:8">
-      <c r="A41" s="5">
-        <v>40</v>
-      </c>
-      <c r="B41" s="5">
-        <v>7</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D41" s="9"/>
-      <c r="E41" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G41" s="8"/>
-      <c r="H41" s="9"/>
-    </row>
-    <row r="42" spans="1:8">
-      <c r="A42" s="5">
-        <v>41</v>
-      </c>
-      <c r="B42" s="5">
-        <v>7</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D42" s="9"/>
-      <c r="E42" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G42" s="8"/>
-      <c r="H42" s="9"/>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="5">
-        <v>42</v>
-      </c>
-      <c r="B43" s="5">
-        <v>7</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D43" s="9"/>
-      <c r="E43" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G43" s="8"/>
-      <c r="H43" s="9"/>
-    </row>
-    <row r="44" spans="1:8">
-      <c r="A44" s="5">
-        <v>43</v>
-      </c>
-      <c r="B44" s="5">
-        <v>8</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D44" s="9"/>
-      <c r="E44" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G44" s="8"/>
-      <c r="H44" s="9"/>
-    </row>
-    <row r="45" spans="1:8">
-      <c r="A45" s="5">
-        <v>44</v>
-      </c>
-      <c r="B45" s="5">
-        <v>8</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D45" s="9"/>
-      <c r="E45" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G45" s="8"/>
-      <c r="H45" s="9"/>
-    </row>
-    <row r="46" spans="1:8">
-      <c r="A46" s="5">
-        <v>45</v>
-      </c>
-      <c r="B46" s="5">
-        <v>8</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D46" s="9"/>
-      <c r="E46" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F46" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G46" s="8"/>
-      <c r="H46" s="9"/>
-    </row>
-    <row r="47" spans="1:8">
-      <c r="A47" s="5">
-        <v>46</v>
-      </c>
-      <c r="B47" s="5">
-        <v>9</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D47" s="9"/>
-      <c r="E47" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="F47" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G47" s="8"/>
-      <c r="H47" s="9"/>
-    </row>
-    <row r="48" spans="1:8">
-      <c r="A48" s="5">
-        <v>47</v>
-      </c>
-      <c r="B48" s="5">
-        <v>9</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D48" s="9"/>
-      <c r="E48" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G48" s="8"/>
-      <c r="H48" s="9"/>
-    </row>
-    <row r="49" spans="1:8">
-      <c r="A49" s="5">
-        <v>48</v>
-      </c>
-      <c r="B49" s="5">
-        <v>10</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D49" s="9"/>
-      <c r="E49" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F49" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G49" s="8"/>
-      <c r="H49" s="9"/>
-    </row>
-    <row r="50" spans="1:8" ht="27">
-      <c r="A50" s="5">
-        <v>49</v>
-      </c>
-      <c r="B50" s="5">
-        <v>10</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D50" s="9"/>
-      <c r="E50" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="8"/>
-      <c r="H50" s="9"/>
-    </row>
-    <row r="51" spans="1:8">
-      <c r="A51" s="5">
-        <v>50</v>
-      </c>
-      <c r="B51" s="5">
-        <v>10</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D51" s="9"/>
-      <c r="E51" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="F51" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G51" s="8"/>
-      <c r="H51" s="9"/>
+      <c r="G51" s="6"/>
+      <c r="H51" s="7"/>
     </row>
     <row r="53" spans="1:8">
-      <c r="A53" s="10" t="s">
+      <c r="A53" s="8" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="54" spans="1:8">
-      <c r="A54" s="2" t="s">
+      <c r="A54" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="2"/>
-      <c r="H54" s="2"/>
+      <c r="B54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19"/>
+      <c r="F54" s="19"/>
+      <c r="G54" s="19"/>
+      <c r="H54" s="19"/>
     </row>
     <row r="55" spans="1:8">
-      <c r="A55" s="1" t="s">
+      <c r="A55" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="1"/>
-      <c r="E55" s="1"/>
-      <c r="F55" s="1"/>
-      <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
+      <c r="B55" s="20"/>
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="20"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="20"/>
+      <c r="H55" s="20"/>
     </row>
     <row r="56" spans="1:8">
-      <c r="A56" s="1" t="s">
+      <c r="A56" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="B56" s="1"/>
-      <c r="C56" s="1"/>
-      <c r="D56" s="1"/>
-      <c r="E56" s="1"/>
-      <c r="F56" s="1"/>
-      <c r="G56" s="1"/>
-      <c r="H56" s="1"/>
+      <c r="B56" s="20"/>
+      <c r="C56" s="20"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="20"/>
+      <c r="F56" s="20"/>
+      <c r="G56" s="20"/>
+      <c r="H56" s="20"/>
     </row>
     <row r="57" spans="1:8">
-      <c r="A57" s="1" t="s">
+      <c r="A57" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="1"/>
-      <c r="E57" s="1"/>
-      <c r="F57" s="1"/>
-      <c r="G57" s="1"/>
-      <c r="H57" s="1"/>
+      <c r="B57" s="20"/>
+      <c r="C57" s="20"/>
+      <c r="D57" s="20"/>
+      <c r="E57" s="20"/>
+      <c r="F57" s="20"/>
+      <c r="G57" s="20"/>
+      <c r="H57" s="20"/>
     </row>
     <row r="58" spans="1:8">
-      <c r="A58" s="1" t="s">
+      <c r="A58" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B58" s="1"/>
-      <c r="C58" s="1"/>
-      <c r="D58" s="1"/>
-      <c r="E58" s="1"/>
-      <c r="F58" s="1"/>
-      <c r="G58" s="1"/>
-      <c r="H58" s="1"/>
+      <c r="B58" s="20"/>
+      <c r="C58" s="20"/>
+      <c r="D58" s="20"/>
+      <c r="E58" s="20"/>
+      <c r="F58" s="20"/>
+      <c r="G58" s="20"/>
+      <c r="H58" s="20"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H51"/>
@@ -5419,260 +5418,260 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="10" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="5">
+      <c r="A2" s="3">
         <v>0</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="3">
         <f>COUNTIF(체크리스트!$B$2:$B$51,A2)</f>
         <v>5</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="3">
         <f>COUNTIFS(체크리스트!$B$2:$B$51,A2,체크리스트!$F$2:$F$51,"완료")</f>
         <v>5</v>
       </c>
-      <c r="E2" s="14">
+      <c r="E2" s="12">
         <f t="shared" ref="E2:E13" si="0">IFERROR(D2/C2,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="5">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="3">
         <f>COUNTIF(체크리스트!$B$2:$B$51,A3)</f>
         <v>9</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="3">
         <f>COUNTIFS(체크리스트!$B$2:$B$51,A3,체크리스트!$F$2:$F$51,"완료")</f>
         <v>8</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="12">
         <f t="shared" si="0"/>
         <v>0.88888888888888884</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="5">
+      <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="3">
         <f>COUNTIF(체크리스트!$B$2:$B$51,A4)</f>
         <v>5</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="3">
         <f>COUNTIFS(체크리스트!$B$2:$B$51,A4,체크리스트!$F$2:$F$51,"완료")</f>
+        <v>5</v>
+      </c>
+      <c r="E4" s="12">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="3">
+        <v>3</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="3">
+        <f>COUNTIF(체크리스트!$B$2:$B$51,A5)</f>
+        <v>5</v>
+      </c>
+      <c r="D5" s="3">
+        <f>COUNTIFS(체크리스트!$B$2:$B$51,A5,체크리스트!$F$2:$F$51,"완료")</f>
         <v>0</v>
       </c>
-      <c r="E4" s="14">
+      <c r="E5" s="12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="5">
-        <v>3</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="5">
-        <f>COUNTIF(체크리스트!$B$2:$B$51,A5)</f>
+    <row r="6" spans="1:5">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="3">
+        <f>COUNTIF(체크리스트!$B$2:$B$51,A6)</f>
         <v>5</v>
       </c>
-      <c r="D5" s="5">
-        <f>COUNTIFS(체크리스트!$B$2:$B$51,A5,체크리스트!$F$2:$F$51,"완료")</f>
+      <c r="D6" s="3">
+        <f>COUNTIFS(체크리스트!$B$2:$B$51,A6,체크리스트!$F$2:$F$51,"완료")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E6" s="12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="5">
+    <row r="7" spans="1:5">
+      <c r="A7" s="3">
+        <v>5</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="3">
+        <f>COUNTIF(체크리스트!$B$2:$B$51,A7)</f>
         <v>4</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" s="5">
-        <f>COUNTIF(체크리스트!$B$2:$B$51,A6)</f>
-        <v>5</v>
-      </c>
-      <c r="D6" s="5">
-        <f>COUNTIFS(체크리스트!$B$2:$B$51,A6,체크리스트!$F$2:$F$51,"완료")</f>
+      <c r="D7" s="3">
+        <f>COUNTIFS(체크리스트!$B$2:$B$51,A7,체크리스트!$F$2:$F$51,"완료")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E7" s="12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="5">
-        <v>5</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="5">
-        <f>COUNTIF(체크리스트!$B$2:$B$51,A7)</f>
+    <row r="8" spans="1:5">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="3">
+        <f>COUNTIF(체크리스트!$B$2:$B$51,A8)</f>
         <v>4</v>
       </c>
-      <c r="D7" s="5">
-        <f>COUNTIFS(체크리스트!$B$2:$B$51,A7,체크리스트!$F$2:$F$51,"완료")</f>
+      <c r="D8" s="3">
+        <f>COUNTIFS(체크리스트!$B$2:$B$51,A8,체크리스트!$F$2:$F$51,"완료")</f>
         <v>0</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E8" s="12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="5">
-        <v>6</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="5">
-        <f>COUNTIF(체크리스트!$B$2:$B$51,A8)</f>
-        <v>4</v>
-      </c>
-      <c r="D8" s="5">
-        <f>COUNTIFS(체크리스트!$B$2:$B$51,A8,체크리스트!$F$2:$F$51,"완료")</f>
+    <row r="9" spans="1:5">
+      <c r="A9" s="3">
+        <v>7</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="3">
+        <f>COUNTIF(체크리스트!$B$2:$B$51,A9)</f>
+        <v>5</v>
+      </c>
+      <c r="D9" s="3">
+        <f>COUNTIFS(체크리스트!$B$2:$B$51,A9,체크리스트!$F$2:$F$51,"완료")</f>
         <v>0</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E9" s="12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="5">
-        <v>7</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="5">
-        <f>COUNTIF(체크리스트!$B$2:$B$51,A9)</f>
-        <v>5</v>
-      </c>
-      <c r="D9" s="5">
-        <f>COUNTIFS(체크리스트!$B$2:$B$51,A9,체크리스트!$F$2:$F$51,"완료")</f>
+    <row r="10" spans="1:5">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="3">
+        <f>COUNTIF(체크리스트!$B$2:$B$51,A10)</f>
+        <v>3</v>
+      </c>
+      <c r="D10" s="3">
+        <f>COUNTIFS(체크리스트!$B$2:$B$51,A10,체크리스트!$F$2:$F$51,"완료")</f>
         <v>0</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E10" s="12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="5">
-        <v>8</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="5">
-        <f>COUNTIF(체크리스트!$B$2:$B$51,A10)</f>
-        <v>3</v>
-      </c>
-      <c r="D10" s="5">
-        <f>COUNTIFS(체크리스트!$B$2:$B$51,A10,체크리스트!$F$2:$F$51,"완료")</f>
+    <row r="11" spans="1:5">
+      <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="3">
+        <f>COUNTIF(체크리스트!$B$2:$B$51,A11)</f>
+        <v>2</v>
+      </c>
+      <c r="D11" s="3">
+        <f>COUNTIFS(체크리스트!$B$2:$B$51,A11,체크리스트!$F$2:$F$51,"완료")</f>
         <v>0</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E11" s="12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="5">
-        <v>9</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="5">
-        <f>COUNTIF(체크리스트!$B$2:$B$51,A11)</f>
-        <v>2</v>
-      </c>
-      <c r="D11" s="5">
-        <f>COUNTIFS(체크리스트!$B$2:$B$51,A11,체크리스트!$F$2:$F$51,"완료")</f>
+    <row r="12" spans="1:5">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="3">
+        <f>COUNTIF(체크리스트!$B$2:$B$51,A12)</f>
+        <v>3</v>
+      </c>
+      <c r="D12" s="3">
+        <f>COUNTIFS(체크리스트!$B$2:$B$51,A12,체크리스트!$F$2:$F$51,"완료")</f>
         <v>0</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E12" s="12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="5">
-        <v>10</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="C12" s="5">
-        <f>COUNTIF(체크리스트!$B$2:$B$51,A12)</f>
-        <v>3</v>
-      </c>
-      <c r="D12" s="5">
-        <f>COUNTIFS(체크리스트!$B$2:$B$51,A12,체크리스트!$F$2:$F$51,"완료")</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="14">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="C13" s="16">
+      <c r="C13" s="14">
         <f>SUM(C2:C12)</f>
         <v>50</v>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="14">
         <f>SUM(D2:D12)</f>
-        <v>13</v>
-      </c>
-      <c r="E13" s="18">
+        <v>18</v>
+      </c>
+      <c r="E13" s="16">
         <f t="shared" si="0"/>
-        <v>0.26</v>
+        <v>0.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: BitCtrl(I2C 비트 타이밍 FSM) RTL 구현 및 TB 뼈대 추가, Phase2~4 설계 문서 정리
- source/BitCtrl.vhd: 2-process 스타일로 비트/START/STOP 파형 생성 FSM 구현
  (WAIT/SCL_LOW/SDA_SETUP/SCL_HIGH/GEN_START/GEN_STOP)
- sim/BitCtrlTb.vhd: BitCtrl 단독 검증용 테스트벤치 뼈대 작성
- 참고사항/Phase2~4 마크다운: 블록다이어그램/비트타이밍차트/FSM 설계 단계별 정리
- BItTxRx_FSM.drawio, ByteData_FSM.drawio, I2CMaster_FSM.drawio: 3계층 FSM 상태전이도 추가
- TpgCtrlTop_Block_Diagram.drawio, 타이밍 계산/비트차트 엑셀: 최신 설계 반영 업데이트

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/참고사항/24LC256_체크리스트_1.xlsx
+++ b/참고사항/24LC256_체크리스트_1.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+  <workbookPr codeName="현재_통합_문서"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BLUE\work\VHDL\FSM_EEPROM\참고사항\"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="90">
   <si>
     <t>No</t>
   </si>
@@ -3224,6 +3224,9 @@
   </si>
   <si>
     <t>24LC256</t>
+  </si>
+  <si>
+    <t>진행중</t>
   </si>
 </sst>
 </file>
@@ -3712,7 +3715,7 @@
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.8</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -3745,11 +3748,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="1354901616"/>
-        <c:axId val="1354900528"/>
+        <c:axId val="1116944208"/>
+        <c:axId val="1116947472"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1354901616"/>
+        <c:axId val="1116944208"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3816,7 +3819,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1354900528"/>
+        <c:crossAx val="1116947472"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3824,7 +3827,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1354900528"/>
+        <c:axId val="1116947472"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3901,7 +3904,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1354901616"/>
+        <c:crossAx val="1116944208"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4217,6 +4220,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:H58"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
@@ -4801,7 +4805,7 @@
         <v>41</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G26" s="6"/>
       <c r="H26" s="7"/>
@@ -4821,7 +4825,7 @@
         <v>42</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G27" s="6"/>
       <c r="H27" s="7"/>
@@ -4841,7 +4845,7 @@
         <v>43</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="7"/>
@@ -4861,7 +4865,7 @@
         <v>44</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="7"/>
@@ -4881,7 +4885,7 @@
         <v>45</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>11</v>
+        <v>89</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="7"/>
@@ -5406,6 +5410,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
@@ -5524,11 +5529,11 @@
       </c>
       <c r="D6" s="3">
         <f>COUNTIFS(체크리스트!$B$2:$B$51,A6,체크리스트!$F$2:$F$51,"완료")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E6" s="12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -5664,11 +5669,11 @@
       </c>
       <c r="D13" s="14">
         <f>SUM(D2:D12)</f>
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E13" s="16">
         <f t="shared" si="0"/>
-        <v>0.42</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>